<commit_message>
added key.properties to .gitignore
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/TestData.xlsx
+++ b/src/test/resources/testData/TestData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/daefa56d07a68b4b/Documents/practise/projects/stripeAPIAutomation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED4C399E-1D77-4FAD-BBEC-688C7E6BFAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{ED4C399E-1D77-4FAD-BBEC-688C7E6BFAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22264591-31FC-4612-A4D7-8A2A81A8B183}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6F6605D0-55CE-43E7-9052-60E05857A033}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="TestDataSheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,16 +39,52 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>testAPI1</t>
+  </si>
+  <si>
+    <t>endOfTestData</t>
+  </si>
+  <si>
+    <t>basePath</t>
+  </si>
+  <si>
+    <t>v1/</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>vijay</t>
+  </si>
+  <si>
+    <t>joshi@hotmail.com</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>3660 james trail drive</t>
+  </si>
+  <si>
+    <t>endPoint</t>
+  </si>
+  <si>
+    <t>customers?limit=3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,13 +98,45 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A00FF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -80,14 +148,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -101,6 +175,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -420,15 +498,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF87677C-6ED9-4338-B081-35BE41D912AE}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>4043699472</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{1A540DE2-5AFE-49AB-B975-98FCBD77126F}"/>
+    <hyperlink ref="C7" r:id="rId2" display="joshi@hotmail.com" xr:uid="{CF883DAC-3A8A-49BB-89ED-5C5425E3A910}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>